<commit_message>
feat: add 50 test products, Category column in Excel, optimizations, and update docs
- Add 50 Indian spice & grocery products to KetanShop.xlsx (56 total)
- Add Category column to KetanShop.xlsx for seed/import categorization
- Add Sharp-based image compression (600px WebP @ 85% quality)
- Add server-side pagination, in-memory cache, 7-day browser cache
- Add infinite scroll with IntersectionObserver + image prefetching
- Add skeleton loading shimmer animations
- Add Lenis smooth scrolling library
- Add React.lazy code splitting for AdminPage
- Add existing categories info message on Excel import page
- Add /api/admin/categories endpoint
- Add scripts/check-db-stats.js and recompress-images.js
- Remove legacy public/product_images/ files (images stored in DB now)
- Update README with all features, optimizations, and 56 product catalog
</commit_message>
<xml_diff>
--- a/KetanShop.xlsx
+++ b/KetanShop.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I57"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -425,6 +425,9 @@
       <c r="H1" t="str">
         <v>Availability</v>
       </c>
+      <c r="I1" t="str">
+        <v>Category</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -448,6 +451,12 @@
       <c r="G2" t="str">
         <v>yes</v>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>Sweets &amp; Snacks</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -468,8 +477,14 @@
       <c r="F3">
         <v>2</v>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
       <c r="H3" t="str">
         <v>yes</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Spices</v>
       </c>
     </row>
     <row r="4">
@@ -491,8 +506,14 @@
       <c r="F4">
         <v>3</v>
       </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
       <c r="H4" t="str">
         <v>yes</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Sweets &amp; Snacks</v>
       </c>
     </row>
     <row r="5">
@@ -514,8 +535,14 @@
       <c r="F5">
         <v>4</v>
       </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
       <c r="H5" t="str">
         <v>yes</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Spices</v>
       </c>
     </row>
     <row r="6">
@@ -537,8 +564,14 @@
       <c r="F6">
         <v>5</v>
       </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
       <c r="H6" t="str">
         <v>yes</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Grains &amp; Rice</v>
       </c>
     </row>
     <row r="7">
@@ -560,13 +593,1469 @@
       <c r="F7">
         <v>6</v>
       </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
       <c r="H7" t="str">
         <v>yes</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Pickles &amp; Chutneys</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Turmeric Powder (Haldi Powder)</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8">
+        <v>60</v>
+      </c>
+      <c r="D8">
+        <v>60</v>
+      </c>
+      <c r="E8" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F8">
+        <v>7</v>
+      </c>
+      <c r="G8" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Red Chili Powder (Lal Mirch)</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9">
+        <v>80</v>
+      </c>
+      <c r="D9">
+        <v>80</v>
+      </c>
+      <c r="E9" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F9">
+        <v>8</v>
+      </c>
+      <c r="G9" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Cumin Seeds (Jeera)</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10">
+        <v>120</v>
+      </c>
+      <c r="D10">
+        <v>120</v>
+      </c>
+      <c r="E10" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F10">
+        <v>9</v>
+      </c>
+      <c r="G10" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Coriander Powder (Dhania Powder)</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11">
+        <v>70</v>
+      </c>
+      <c r="D11">
+        <v>70</v>
+      </c>
+      <c r="E11" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F11">
+        <v>10</v>
+      </c>
+      <c r="G11" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Garam Masala</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12">
+        <v>90</v>
+      </c>
+      <c r="D12">
+        <v>90</v>
+      </c>
+      <c r="E12" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F12">
+        <v>11</v>
+      </c>
+      <c r="G12" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Black Pepper (Kali Mirch)</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13">
+        <v>250</v>
+      </c>
+      <c r="D13">
+        <v>250</v>
+      </c>
+      <c r="E13" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F13">
+        <v>12</v>
+      </c>
+      <c r="G13" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Green Cardamom (Elaichi)</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14">
+        <v>350</v>
+      </c>
+      <c r="D14">
+        <v>350</v>
+      </c>
+      <c r="E14" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F14">
+        <v>13</v>
+      </c>
+      <c r="G14" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Cloves (Laung)</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15">
+        <v>320</v>
+      </c>
+      <c r="D15">
+        <v>320</v>
+      </c>
+      <c r="E15" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F15">
+        <v>14</v>
+      </c>
+      <c r="G15" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Cinnamon Sticks (Dalchini)</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16">
+        <v>180</v>
+      </c>
+      <c r="D16">
+        <v>180</v>
+      </c>
+      <c r="E16" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F16">
+        <v>15</v>
+      </c>
+      <c r="G16" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Mustard Seeds (Rai/Sarson)</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17">
+        <v>60</v>
+      </c>
+      <c r="D17">
+        <v>60</v>
+      </c>
+      <c r="E17" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F17">
+        <v>16</v>
+      </c>
+      <c r="G17" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Fennel Seeds (Saunf)</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18">
+        <v>80</v>
+      </c>
+      <c r="D18">
+        <v>80</v>
+      </c>
+      <c r="E18" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F18">
+        <v>17</v>
+      </c>
+      <c r="G18" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Fenugreek Seeds (Methi)</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19">
+        <v>55</v>
+      </c>
+      <c r="D19">
+        <v>55</v>
+      </c>
+      <c r="E19" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F19">
+        <v>18</v>
+      </c>
+      <c r="G19" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Asafoetida (Hing)</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20">
+        <v>150</v>
+      </c>
+      <c r="D20">
+        <v>150</v>
+      </c>
+      <c r="E20" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F20">
+        <v>19</v>
+      </c>
+      <c r="G20" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Dry Mango Powder (Amchur)</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21">
+        <v>140</v>
+      </c>
+      <c r="D21">
+        <v>140</v>
+      </c>
+      <c r="E21" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F21">
+        <v>20</v>
+      </c>
+      <c r="G21" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Pomegranate Seed Powder (Anardana)</v>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22">
+        <v>180</v>
+      </c>
+      <c r="D22">
+        <v>180</v>
+      </c>
+      <c r="E22" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F22">
+        <v>21</v>
+      </c>
+      <c r="G22" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Saffron (Kesar)</v>
+      </c>
+      <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23">
+        <v>800</v>
+      </c>
+      <c r="D23">
+        <v>800</v>
+      </c>
+      <c r="E23" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F23">
+        <v>22</v>
+      </c>
+      <c r="G23" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Nutmeg (Jaiphal)</v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24">
+        <v>200</v>
+      </c>
+      <c r="D24">
+        <v>200</v>
+      </c>
+      <c r="E24" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F24">
+        <v>23</v>
+      </c>
+      <c r="G24" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Mace (Javitri)</v>
+      </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25">
+        <v>280</v>
+      </c>
+      <c r="D25">
+        <v>280</v>
+      </c>
+      <c r="E25" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F25">
+        <v>24</v>
+      </c>
+      <c r="G25" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Curry Leaves Powder (Kadi Patta)</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26">
+        <v>100</v>
+      </c>
+      <c r="D26">
+        <v>100</v>
+      </c>
+      <c r="E26" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F26">
+        <v>25</v>
+      </c>
+      <c r="G26" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Goda Masala (Kolhapuri)</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27">
+        <v>120</v>
+      </c>
+      <c r="D27">
+        <v>120</v>
+      </c>
+      <c r="E27" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F27">
+        <v>26</v>
+      </c>
+      <c r="G27" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v>Spices</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Sonam Masoori Rice</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28">
+        <v>160</v>
+      </c>
+      <c r="D28">
+        <v>160</v>
+      </c>
+      <c r="E28" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F28">
+        <v>27</v>
+      </c>
+      <c r="G28" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Brown Rice</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29">
+        <v>180</v>
+      </c>
+      <c r="D29">
+        <v>180</v>
+      </c>
+      <c r="E29" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F29">
+        <v>28</v>
+      </c>
+      <c r="G29" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Toor Dal (Arhar Dal)</v>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30">
+        <v>150</v>
+      </c>
+      <c r="D30">
+        <v>150</v>
+      </c>
+      <c r="E30" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F30">
+        <v>29</v>
+      </c>
+      <c r="G30" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Moong Dal (Green Gram)</v>
+      </c>
+      <c r="B31" t="str">
+        <v/>
+      </c>
+      <c r="C31">
+        <v>130</v>
+      </c>
+      <c r="D31">
+        <v>130</v>
+      </c>
+      <c r="E31" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F31">
+        <v>30</v>
+      </c>
+      <c r="G31" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
+      <c r="I31" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Chana Dal (Bengal Gram)</v>
+      </c>
+      <c r="B32" t="str">
+        <v/>
+      </c>
+      <c r="C32">
+        <v>110</v>
+      </c>
+      <c r="D32">
+        <v>110</v>
+      </c>
+      <c r="E32" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F32">
+        <v>31</v>
+      </c>
+      <c r="G32" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Urad Dal (Black Gram)</v>
+      </c>
+      <c r="B33" t="str">
+        <v/>
+      </c>
+      <c r="C33">
+        <v>140</v>
+      </c>
+      <c r="D33">
+        <v>140</v>
+      </c>
+      <c r="E33" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F33">
+        <v>32</v>
+      </c>
+      <c r="G33" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Masoor Dal (Red Lentil)</v>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34">
+        <v>120</v>
+      </c>
+      <c r="D34">
+        <v>120</v>
+      </c>
+      <c r="E34" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F34">
+        <v>33</v>
+      </c>
+      <c r="G34" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Whole Wheat Flour (Atta)</v>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35">
+        <v>45</v>
+      </c>
+      <c r="D35">
+        <v>45</v>
+      </c>
+      <c r="E35" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F35">
+        <v>34</v>
+      </c>
+      <c r="G35" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
+      <c r="I35" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Besan (Gram Flour)</v>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36">
+        <v>70</v>
+      </c>
+      <c r="D36">
+        <v>70</v>
+      </c>
+      <c r="E36" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F36">
+        <v>35</v>
+      </c>
+      <c r="G36" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Rice Flour (Chawal ka Atta)</v>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37">
+        <v>65</v>
+      </c>
+      <c r="D37">
+        <v>65</v>
+      </c>
+      <c r="E37" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F37">
+        <v>36</v>
+      </c>
+      <c r="G37" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Jowar Flour (Sorghum)</v>
+      </c>
+      <c r="B38" t="str">
+        <v/>
+      </c>
+      <c r="C38">
+        <v>55</v>
+      </c>
+      <c r="D38">
+        <v>55</v>
+      </c>
+      <c r="E38" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F38">
+        <v>37</v>
+      </c>
+      <c r="G38" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Bajra Flour (Millet)</v>
+      </c>
+      <c r="B39" t="str">
+        <v/>
+      </c>
+      <c r="C39">
+        <v>50</v>
+      </c>
+      <c r="D39">
+        <v>50</v>
+      </c>
+      <c r="E39" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F39">
+        <v>38</v>
+      </c>
+      <c r="G39" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Ragi Flour (Finger Millet)</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40">
+        <v>80</v>
+      </c>
+      <c r="D40">
+        <v>80</v>
+      </c>
+      <c r="E40" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F40">
+        <v>39</v>
+      </c>
+      <c r="G40" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Poha (Flattened Rice)</v>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41">
+        <v>55</v>
+      </c>
+      <c r="D41">
+        <v>55</v>
+      </c>
+      <c r="E41" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F41">
+        <v>40</v>
+      </c>
+      <c r="G41" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v>Grains &amp; Rice</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Cow Ghee (Gau Tup)</v>
+      </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42">
+        <v>550</v>
+      </c>
+      <c r="D42">
+        <v>550</v>
+      </c>
+      <c r="E42" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F42">
+        <v>41</v>
+      </c>
+      <c r="G42" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
+      <c r="I42" t="str">
+        <v>Oils &amp; Ghee</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Kachi Ghani Mustard Oil</v>
+      </c>
+      <c r="B43" t="str">
+        <v/>
+      </c>
+      <c r="C43">
+        <v>220</v>
+      </c>
+      <c r="D43">
+        <v>220</v>
+      </c>
+      <c r="E43" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F43">
+        <v>42</v>
+      </c>
+      <c r="G43" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
+      <c r="I43" t="str">
+        <v>Oils &amp; Ghee</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Peanut Oil (Groundnut Oil)</v>
+      </c>
+      <c r="B44" t="str">
+        <v/>
+      </c>
+      <c r="C44">
+        <v>200</v>
+      </c>
+      <c r="D44">
+        <v>200</v>
+      </c>
+      <c r="E44" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F44">
+        <v>43</v>
+      </c>
+      <c r="G44" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
+      <c r="I44" t="str">
+        <v>Oils &amp; Ghee</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Coconut Oil</v>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45">
+        <v>280</v>
+      </c>
+      <c r="D45">
+        <v>280</v>
+      </c>
+      <c r="E45" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F45">
+        <v>44</v>
+      </c>
+      <c r="G45" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
+      <c r="I45" t="str">
+        <v>Oils &amp; Ghee</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Sunflower Oil</v>
+      </c>
+      <c r="B46" t="str">
+        <v/>
+      </c>
+      <c r="C46">
+        <v>180</v>
+      </c>
+      <c r="D46">
+        <v>180</v>
+      </c>
+      <c r="E46" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F46">
+        <v>45</v>
+      </c>
+      <c r="G46" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H46" t="str">
+        <v/>
+      </c>
+      <c r="I46" t="str">
+        <v>Oils &amp; Ghee</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Til Ladoo (Sesame Ladoo)</v>
+      </c>
+      <c r="B47" t="str">
+        <v/>
+      </c>
+      <c r="C47">
+        <v>120</v>
+      </c>
+      <c r="D47">
+        <v>120</v>
+      </c>
+      <c r="E47" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F47">
+        <v>46</v>
+      </c>
+      <c r="G47" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
+      <c r="I47" t="str">
+        <v>Sweets &amp; Snacks</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Besan Ladoo</v>
+      </c>
+      <c r="B48" t="str">
+        <v/>
+      </c>
+      <c r="C48">
+        <v>180</v>
+      </c>
+      <c r="D48">
+        <v>180</v>
+      </c>
+      <c r="E48" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F48">
+        <v>47</v>
+      </c>
+      <c r="G48" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
+      <c r="I48" t="str">
+        <v>Sweets &amp; Snacks</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Chakli (Murukku)</v>
+      </c>
+      <c r="B49" t="str">
+        <v/>
+      </c>
+      <c r="C49">
+        <v>100</v>
+      </c>
+      <c r="D49">
+        <v>100</v>
+      </c>
+      <c r="E49" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F49">
+        <v>48</v>
+      </c>
+      <c r="G49" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
+      <c r="I49" t="str">
+        <v>Sweets &amp; Snacks</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Bhakarwadi</v>
+      </c>
+      <c r="B50" t="str">
+        <v/>
+      </c>
+      <c r="C50">
+        <v>140</v>
+      </c>
+      <c r="D50">
+        <v>140</v>
+      </c>
+      <c r="E50" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F50">
+        <v>49</v>
+      </c>
+      <c r="G50" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H50" t="str">
+        <v/>
+      </c>
+      <c r="I50" t="str">
+        <v>Sweets &amp; Snacks</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Shankarpali</v>
+      </c>
+      <c r="B51" t="str">
+        <v/>
+      </c>
+      <c r="C51">
+        <v>90</v>
+      </c>
+      <c r="D51">
+        <v>90</v>
+      </c>
+      <c r="E51" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F51">
+        <v>50</v>
+      </c>
+      <c r="G51" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v>Sweets &amp; Snacks</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Lemon Pickle (Nimbu ka Achar)</v>
+      </c>
+      <c r="B52" t="str">
+        <v/>
+      </c>
+      <c r="C52">
+        <v>100</v>
+      </c>
+      <c r="D52">
+        <v>100</v>
+      </c>
+      <c r="E52" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F52">
+        <v>51</v>
+      </c>
+      <c r="G52" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
+      <c r="I52" t="str">
+        <v>Pickles &amp; Chutneys</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Mixed Vegetable Pickle</v>
+      </c>
+      <c r="B53" t="str">
+        <v/>
+      </c>
+      <c r="C53">
+        <v>120</v>
+      </c>
+      <c r="D53">
+        <v>120</v>
+      </c>
+      <c r="E53" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F53">
+        <v>52</v>
+      </c>
+      <c r="G53" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v>Pickles &amp; Chutneys</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Garlic Pickle (Lasunacha Achar)</v>
+      </c>
+      <c r="B54" t="str">
+        <v/>
+      </c>
+      <c r="C54">
+        <v>150</v>
+      </c>
+      <c r="D54">
+        <v>150</v>
+      </c>
+      <c r="E54" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F54">
+        <v>53</v>
+      </c>
+      <c r="G54" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v>Pickles &amp; Chutneys</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Green Chili Pickle (Hari Mirch)</v>
+      </c>
+      <c r="B55" t="str">
+        <v/>
+      </c>
+      <c r="C55">
+        <v>130</v>
+      </c>
+      <c r="D55">
+        <v>130</v>
+      </c>
+      <c r="E55" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F55">
+        <v>54</v>
+      </c>
+      <c r="G55" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v>Pickles &amp; Chutneys</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Dry Coconut Chutney (Sukha Nariyal)</v>
+      </c>
+      <c r="B56" t="str">
+        <v/>
+      </c>
+      <c r="C56">
+        <v>80</v>
+      </c>
+      <c r="D56">
+        <v>80</v>
+      </c>
+      <c r="E56" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F56">
+        <v>55</v>
+      </c>
+      <c r="G56" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v>Pickles &amp; Chutneys</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Masala Chai (Spiced Tea)</v>
+      </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57">
+        <v>250</v>
+      </c>
+      <c r="D57">
+        <v>250</v>
+      </c>
+      <c r="E57" t="str">
+        <v>TBC</v>
+      </c>
+      <c r="F57">
+        <v>56</v>
+      </c>
+      <c r="G57" t="str">
+        <v>yes</v>
+      </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v>Beverages</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I57"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>